<commit_message>
Add PDF export, spanwise plot improvements, warning popups, and optimizer fixes
- export_pdf action: 5-page PDF report (summary table, mass budget pie, spanwise distributions, motor curve, BEMT health bar chart) via matplotlib PdfPages
- plot_spanwise: chord Y-axis starts from 0; vertical r_root line marks structural/aero boundary; horizontal eff_min_chord line shows design floor
- _check_final_warnings: post-optimization popup for negative thrust/torque and bound-active conditions
- SLSQP eps=1e-2 and x0 RPM fix (correct radius for initial tip speed), maxiter=60
- Pre-stall L/D argmax in airfoil.py restricts optimal-alpha search to below CL_max
- mission.xlsx weights updated: w_mass=0.0, w_power=0.5, w_endurance=0.5

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/mission.xlsx
+++ b/data/input/mission.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3072" yWindow="3072" windowWidth="30960" windowHeight="12120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mission" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,7 +25,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -38,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +60,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -423,7 +424,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -520,7 +521,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -593,7 +594,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>target_endurance_min</t>
+          <t>min_endurance_min</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -606,7 +607,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hover endurance target -- drives battery sizing</t>
+          <t>Minimum required hover endurance [min]; battery sized as floor, w_endurance drives above it</t>
         </is>
       </c>
     </row>
@@ -617,7 +618,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -637,7 +638,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -657,7 +658,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>

</xml_diff>